<commit_message>
Added few more test cases
</commit_message>
<xml_diff>
--- a/src/test/resources/dataFiles/excelFiles/balanceMissingOrInconsistentWithStatus.xlsx
+++ b/src/test/resources/dataFiles/excelFiles/balanceMissingOrInconsistentWithStatus.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Java\blocrecon\src\test\resources\dataFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Java\blocrecon\src\test\resources\dataFiles\excelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{392252C1-9D8B-488D-81B6-917B767F66D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36B75FDE-3CFC-46B1-8C0E-B142F8DE59F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{CA011A21-70A2-4DF5-AE26-B4AB6324FE8A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{CA011A21-70A2-4DF5-AE26-B4AB6324FE8A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>